<commit_message>
Update final evaluation CSVs and compiled Excel sheets with newly trained adapted models
</commit_message>
<xml_diff>
--- a/experiments/Performance_result.xlsx
+++ b/experiments/Performance_result.xlsx
@@ -372,7 +372,7 @@
         <v>0.6204</v>
       </c>
       <c r="E11" t="n">
-        <v>8.1364</v>
+        <v>7.9861</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -392,14 +392,14 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.6519</v>
+        <v>0.863</v>
       </c>
       <c r="E12" t="n">
-        <v>7.0601</v>
+        <v>7.4261</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1408/2160</t>
+          <t>1864/2160</t>
         </is>
       </c>
     </row>
@@ -415,14 +415,14 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.5796</v>
+        <v>0.6935</v>
       </c>
       <c r="E13" t="n">
-        <v>6.9941</v>
+        <v>6.596</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1252/2160</t>
+          <t>1498/2160</t>
         </is>
       </c>
     </row>
@@ -441,7 +441,7 @@
         <v>0.5444</v>
       </c>
       <c r="E14" t="n">
-        <v>13.7299</v>
+        <v>13.2994</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -506,23 +506,23 @@
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>j-hartmann/emotion-english-distilroberta-base</t>
+          <t>chase1zhang/youtube-emotion-jhartmann-distilroberta-domain-adapted</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>seven-emotion classification</t>
+          <t>YouTube-domain adapted DistilRoBERTa</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.409</v>
+        <v>0.8</v>
       </c>
       <c r="E21" t="n">
-        <v>9.716900000000001</v>
+        <v>9.532400000000001</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>409/1000</t>
+          <t>800/1000</t>
         </is>
       </c>
     </row>
@@ -538,14 +538,14 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.467</v>
+        <v>0.405</v>
       </c>
       <c r="E22" t="n">
-        <v>9.448499999999999</v>
+        <v>10.4224</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>467/1000</t>
+          <t>405/1000</t>
         </is>
       </c>
     </row>
@@ -561,37 +561,37 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.665</v>
+        <v>0.83</v>
       </c>
       <c r="E23" t="n">
-        <v>9.4885</v>
+        <v>9.3592</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>665/1000</t>
+          <t>830/1000</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" t="inlineStr">
         <is>
-          <t>SamLowe/roberta-base-go_emotions</t>
+          <t>chase1zhang/youtube-emotion-samlowe-roberta-domain-adapted</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>seven-emotion classification</t>
+          <t>YouTube-domain adapted RoBERTa</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.443</v>
+        <v>0.842</v>
       </c>
       <c r="E24" t="n">
-        <v>19.3556</v>
+        <v>19.0029</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>443/1000</t>
+          <t>842/1000</t>
         </is>
       </c>
     </row>
@@ -610,7 +610,7 @@
         <v>0.456</v>
       </c>
       <c r="E25" t="n">
-        <v>69.09010000000001</v>
+        <v>69.0069</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -633,7 +633,7 @@
         <v>0.597</v>
       </c>
       <c r="E26" t="n">
-        <v>19.179</v>
+        <v>18.01</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -656,7 +656,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>chase1zhang/youtube-emotion-distilbert-domain-adapted</t>
+          <t>chase1zhang/youtube-emotion-samlowe-roberta-domain-adapted</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>It is project-owned, compact for Streamlit deployment, and has the best current YouTube-domain validation accuracy (0.6650).</t>
+          <t>It is project-owned, compact for Streamlit deployment, and has the best current YouTube-domain validation accuracy (0.8420).</t>
         </is>
       </c>
     </row>
@@ -765,7 +765,7 @@
     <row r="41">
       <c r="B41" t="inlineStr">
         <is>
-          <t>Pre-tuning baseline</t>
+          <t>YouTube-domain adapted DistilRoBERTa (j-hartmann)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -782,7 +782,7 @@
         <v>0.4467</v>
       </c>
       <c r="F41" t="n">
-        <v>1.0456</v>
+        <v>0.979</v>
       </c>
     </row>
     <row r="42">
@@ -805,7 +805,7 @@
         <v>0.4667</v>
       </c>
       <c r="F42" t="n">
-        <v>0.8745000000000001</v>
+        <v>0.8515</v>
       </c>
     </row>
     <row r="43">
@@ -828,13 +828,13 @@
         <v>0.4733</v>
       </c>
       <c r="F43" t="n">
-        <v>0.916</v>
+        <v>0.8547</v>
       </c>
     </row>
     <row r="44">
       <c r="B44" t="inlineStr">
         <is>
-          <t>Public GoEmotions RoBERTa (SamLowe)</t>
+          <t>YouTube-domain adapted RoBERTa (SamLowe)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -851,7 +851,7 @@
         <v>0.5333</v>
       </c>
       <c r="F44" t="n">
-        <v>1.9613</v>
+        <v>1.9588</v>
       </c>
     </row>
     <row r="45">
@@ -874,7 +874,7 @@
         <v>0.4133</v>
       </c>
       <c r="F45" t="n">
-        <v>6.8888</v>
+        <v>6.8108</v>
       </c>
     </row>
     <row r="46">
@@ -897,7 +897,7 @@
         <v>0.7</v>
       </c>
       <c r="F46" t="n">
-        <v>1.9177</v>
+        <v>1.8761</v>
       </c>
     </row>
     <row r="50">

</xml_diff>

<commit_message>
Add DeepSeek AI labeling, Pipeline 3 business decision engine, and 3 sentiment model comparison
- Streamlit: replace sentiment text_input with selectbox (CardiffNLP/lxyuan/FiniteAutomata)
- Pipeline 3: rule-based business decision engine combining emotion + sentiment predictions
- Excel: add 3 sentiment model metrics and Pipeline 3 decision rules to Performance_result.xlsx
- Reports: add Pipeline 3 section, 3-model sentiment comparison tables (CN + EN)
- DeepSeek labeling: new script to label 8,000 YouTube comments via DeepSeek API
- Training data: build balanced train/validation splits from DeepSeek labels
- Benchmark: expand script for 150->500 comments with DeepSeek labeling
- Notebook: update Colab training to use DeepSeek-labeled data
- Dependencies: add openai>=1.0

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/Performance_result.xlsx
+++ b/experiments/Performance_result.xlsx
@@ -2,10 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21400" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
     <sheet name="Performance" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -27,7 +31,13 @@
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -36,8 +46,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -251,6 +262,8 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -260,8 +273,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F57"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:G67"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col width="43" customWidth="1" min="2" max="6"/>
+  </cols>
   <sheetData>
     <row r="2">
       <c r="B2" t="inlineStr">
@@ -372,7 +388,7 @@
         <v>0.6204</v>
       </c>
       <c r="E11" t="n">
-        <v>7.9861</v>
+        <v>7.2715</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -395,7 +411,7 @@
         <v>0.863</v>
       </c>
       <c r="E12" t="n">
-        <v>7.4261</v>
+        <v>6.9104</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -418,7 +434,7 @@
         <v>0.6935</v>
       </c>
       <c r="E13" t="n">
-        <v>6.596</v>
+        <v>7.0058</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -441,7 +457,7 @@
         <v>0.5444</v>
       </c>
       <c r="E14" t="n">
-        <v>13.2994</v>
+        <v>14.2865</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -518,7 +534,7 @@
         <v>0.8</v>
       </c>
       <c r="E21" t="n">
-        <v>9.532400000000001</v>
+        <v>9.357900000000001</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -541,7 +557,7 @@
         <v>0.405</v>
       </c>
       <c r="E22" t="n">
-        <v>10.4224</v>
+        <v>10.3628</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -564,7 +580,7 @@
         <v>0.83</v>
       </c>
       <c r="E23" t="n">
-        <v>9.3592</v>
+        <v>9.5097</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -587,7 +603,7 @@
         <v>0.842</v>
       </c>
       <c r="E24" t="n">
-        <v>19.0029</v>
+        <v>18.6446</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -610,7 +626,7 @@
         <v>0.456</v>
       </c>
       <c r="E25" t="n">
-        <v>69.0069</v>
+        <v>68.48520000000001</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -633,7 +649,7 @@
         <v>0.597</v>
       </c>
       <c r="E26" t="n">
-        <v>18.01</v>
+        <v>18.5965</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -782,7 +798,7 @@
         <v>0.4467</v>
       </c>
       <c r="F41" t="n">
-        <v>0.979</v>
+        <v>1.0414</v>
       </c>
     </row>
     <row r="42">
@@ -805,7 +821,7 @@
         <v>0.4667</v>
       </c>
       <c r="F42" t="n">
-        <v>0.8515</v>
+        <v>0.8977000000000001</v>
       </c>
     </row>
     <row r="43">
@@ -828,7 +844,7 @@
         <v>0.4733</v>
       </c>
       <c r="F43" t="n">
-        <v>0.8547</v>
+        <v>0.8952</v>
       </c>
     </row>
     <row r="44">
@@ -851,7 +867,7 @@
         <v>0.5333</v>
       </c>
       <c r="F44" t="n">
-        <v>1.9588</v>
+        <v>1.8465</v>
       </c>
     </row>
     <row r="45">
@@ -874,7 +890,7 @@
         <v>0.4133</v>
       </c>
       <c r="F45" t="n">
-        <v>6.8108</v>
+        <v>6.463</v>
       </c>
     </row>
     <row r="46">
@@ -897,7 +913,7 @@
         <v>0.7</v>
       </c>
       <c r="F46" t="n">
-        <v>1.8761</v>
+        <v>1.9316</v>
       </c>
     </row>
     <row r="50">
@@ -959,17 +975,305 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>lxyuan/distilbert-base-multilingual-cased-sentiments-student</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>3-sentiment</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>94/150</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>0.6267</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Fast CPU inference; multilingual support.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>finiteautomata/bertweet-base-sentiment-analysis</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>3-sentiment</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>0/150</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>BERTweet trained on 40k tweets; robust on social media text.</t>
+        </is>
+      </c>
+    </row>
     <row r="56">
       <c r="B56" t="inlineStr">
         <is>
-          <t>Next TODO</t>
+          <t>Pipeline 3 - Business Decision Engine (combining emotion and sentiment)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="B57" t="inlineStr">
         <is>
-          <t>Fine-tune every seven-emotion baseline on the same YouTube-domain training split, then compare original vs adapted models on GoEmotions test, YouTube-domain validation, and the 150-comment app benchmark.</t>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Condition</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Risk Level</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>High Risk</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Negative emotion ratio &gt;= 40% OR Negative sentiment ratio &gt;= 40%</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Review before scaling</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Low Risk</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Dominant emotion is Joy/Surprise AND Positive sentiment ratio &gt;= 50%</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Scale positive creative</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Medium Risk (engagement)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Dominant emotion is Neutral</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Improve engagement hook</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Medium Risk (mixed)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>All other mixed signals</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Monitor and review samples</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Sample Decision Outputs (150-comment app benchmark)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Dominant Emotion</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Neg Emotion %</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Pos Sentiment %</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>d2dgJGkw5p0</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>32.0%</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>22.0%</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Improve engagement hook</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>M8To7iorkxQ</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>joy</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>8.0%</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>74.0%</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Scale positive creative</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>-_-eIVAX1yQ</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>anger</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>68.0%</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>18.0%</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Review before scaling</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
benchmark: evaluate all 8 emotion + 3 sentiment models on 3 datasets
Added RoBERTa-large domain-adapted model to evaluation pipeline.
Results on 150-comment manual benchmark:
- RoBERTa-large adapted: 0.6267 (best)
- RoBERTa adapted: 0.6200
- DistilBERT adapted: 0.5600
- DistilRoBERTa adapted: 0.5533

YouTube-domain validation (798 samples):
- RoBERTa-large adapted: 0.6717 (best)
- RoBERTa adapted: 0.6504
- DistilRoBERTa adapted: 0.6291
- DistilBERT adapted: 0.6028

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/Performance_result.xlsx
+++ b/experiments/Performance_result.xlsx
@@ -388,7 +388,7 @@
         <v>0.6204</v>
       </c>
       <c r="E11" t="n">
-        <v>7.2715</v>
+        <v>7.9813</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -411,7 +411,7 @@
         <v>0.863</v>
       </c>
       <c r="E12" t="n">
-        <v>6.9104</v>
+        <v>6.7953</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -431,14 +431,14 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.6935</v>
+        <v>0.4944</v>
       </c>
       <c r="E13" t="n">
-        <v>7.0058</v>
+        <v>6.7179</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1498/2160</t>
+          <t>1068/2160</t>
         </is>
       </c>
     </row>
@@ -457,7 +457,7 @@
         <v>0.5444</v>
       </c>
       <c r="E14" t="n">
-        <v>14.2865</v>
+        <v>14.2331</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -531,14 +531,14 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.8</v>
+        <v>0.6291</v>
       </c>
       <c r="E21" t="n">
-        <v>9.357900000000001</v>
+        <v>6.662</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>800/1000</t>
+          <t>502/798</t>
         </is>
       </c>
     </row>
@@ -554,14 +554,14 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.405</v>
+        <v>0.3985</v>
       </c>
       <c r="E22" t="n">
-        <v>10.3628</v>
+        <v>6.3273</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>405/1000</t>
+          <t>318/798</t>
         </is>
       </c>
     </row>
@@ -577,14 +577,14 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.83</v>
+        <v>0.6028</v>
       </c>
       <c r="E23" t="n">
-        <v>9.5097</v>
+        <v>6.4113</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>830/1000</t>
+          <t>481/798</t>
         </is>
       </c>
     </row>
@@ -600,37 +600,37 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.842</v>
+        <v>0.6504</v>
       </c>
       <c r="E24" t="n">
-        <v>18.6446</v>
+        <v>13.444</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>842/1000</t>
+          <t>519/798</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
-          <t>j-hartmann/emotion-english-roberta-large</t>
+          <t>chase1zhang/youtube-emotion-roberta-large-domain-adapted</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>seven-emotion classification</t>
+          <t>YouTube-domain adapted RoBERTa-large</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.456</v>
+        <v>0.6717</v>
       </c>
       <c r="E25" t="n">
-        <v>68.48520000000001</v>
+        <v>46.21</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>456/1000</t>
+          <t>536/798</t>
         </is>
       </c>
     </row>
@@ -646,14 +646,14 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.597</v>
+        <v>0.7018</v>
       </c>
       <c r="E26" t="n">
-        <v>18.5965</v>
+        <v>12.6901</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>597/1000</t>
+          <t>560/798</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>It is project-owned, compact for Streamlit deployment, and has the best current YouTube-domain validation accuracy (0.8420).</t>
+          <t>It is project-owned, compact for Streamlit deployment, and has the best current YouTube-domain validation accuracy (0.6504).</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
         <v>0.4467</v>
       </c>
       <c r="F41" t="n">
-        <v>1.0414</v>
+        <v>1.0381</v>
       </c>
     </row>
     <row r="42">
@@ -821,7 +821,7 @@
         <v>0.4667</v>
       </c>
       <c r="F42" t="n">
-        <v>0.8977000000000001</v>
+        <v>0.8488</v>
       </c>
     </row>
     <row r="43">
@@ -844,7 +844,7 @@
         <v>0.4733</v>
       </c>
       <c r="F43" t="n">
-        <v>0.8952</v>
+        <v>0.9343</v>
       </c>
     </row>
     <row r="44">
@@ -867,13 +867,13 @@
         <v>0.5333</v>
       </c>
       <c r="F44" t="n">
-        <v>1.8465</v>
+        <v>2.0179</v>
       </c>
     </row>
     <row r="45">
       <c r="B45" t="inlineStr">
         <is>
-          <t>Public RoBERTa-large 7-emotion</t>
+          <t>YouTube-domain adapted RoBERTa-large (j-hartmann)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -890,7 +890,7 @@
         <v>0.4133</v>
       </c>
       <c r="F45" t="n">
-        <v>6.463</v>
+        <v>7.3825</v>
       </c>
     </row>
     <row r="46">
@@ -913,7 +913,7 @@
         <v>0.7</v>
       </c>
       <c r="F46" t="n">
-        <v>1.9316</v>
+        <v>2.0197</v>
       </c>
     </row>
     <row r="50">

</xml_diff>